<commit_message>
Remove unwanted files, and add AI-summary and text-to-speech
</commit_message>
<xml_diff>
--- a/sent_emails.xlsx
+++ b/sent_emails.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -671,6 +671,60 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-10 22:17:46</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>devanshmalhotra17@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ji</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Jill</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-10 22:17:52</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>devanshmalhotra17@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ji</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Jill</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>